<commit_message>
feat: update timetable generator with AICTE workload calibration, interactive viewer enhancements, and complete export suite
</commit_message>
<xml_diff>
--- a/Teacher_Workload_Sheet.xlsx
+++ b/Teacher_Workload_Sheet.xlsx
@@ -29,28 +29,28 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F4E79"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00595959"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -74,8 +74,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-        <bgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00F9FAFB"/>
+        <bgColor rgb="00F9FAFB"/>
       </patternFill>
     </fill>
     <fill>
@@ -546,45 +546,46 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="45" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
     <col width="35" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>COLLEGE OF ENGINEERING - FACULTY WORKLOAD DISTRIBUTION SHEET</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Weekly Teaching Load Summary (Monday - Saturday) | ISE &amp; CSBS Departments</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
+          <t>Weekly Workload Norms (Prof: 12h, Assoc Prof: 14h, Asst Prof: 16h) | 1 Lab/Section/Week | ISE &amp; CSBS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Sl No</t>
@@ -602,76 +603,81 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Total Hours</t>
+          <t>Target (Hrs)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
+          <t>Assigned (Hrs)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>Theory (Hrs)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Lab (Sessions)</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Lab (Hrs)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>OE (Hrs)</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>PE (Hrs)</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Assigned Subjects</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>Assigned Sections</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
@@ -686,135 +692,141 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>15</v>
+        <v>12</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>12</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P5" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t>Computer Networks, Data Structures Lab, Mathematics for Computing</t>
+        </is>
+      </c>
+      <c r="R5" s="8" t="inlineStr">
+        <is>
+          <t>CSBS_S3_A, ISE_S3_A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Professor 2</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="J5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="K5" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="L5" s="5" t="n">
+      <c r="L6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="M5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="N5" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="O5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Data Visualization, Machine Learning, Physical Education</t>
-        </is>
-      </c>
-      <c r="Q5" s="8" t="inlineStr">
-        <is>
-          <t>CSBS_S5_A, ISE_S5_A, ISE_S5_A,CSBS_S5_A, ISE_S5_B</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>Professor 2</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="O6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="12" t="inlineStr">
+        <is>
+          <t>Computer Networks, Discrete Mathematics, Programming Fundamentals</t>
+        </is>
+      </c>
+      <c r="R6" s="12" t="inlineStr">
+        <is>
+          <t>CSBS_S1_A, CSBS_S1_B, ISE_S3_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Professor 3</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Professor</t>
         </is>
       </c>
-      <c r="D6" s="11" t="n">
-        <v>14</v>
-      </c>
-      <c r="E6" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="F6" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="K6" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="N6" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="P6" s="12" t="inlineStr">
-        <is>
-          <t>Computer Organization, Data Structures Lab, Programming Fundamentals</t>
-        </is>
-      </c>
-      <c r="Q6" s="12" t="inlineStr">
-        <is>
-          <t>CSBS_S1_A, CSBS_S1_B, ISE_S3_B</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Professor 3</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Professor</t>
-        </is>
-      </c>
       <c r="D7" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>18</v>
+        <v>12</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>12</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>0</v>
@@ -826,35 +838,38 @@
         <v>0</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="P7" s="8" t="inlineStr">
-        <is>
-          <t>Data Structures, Digital Logic, Operating Systems</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>CSBS_S1_A, CSBS_S3_B, ISE_S3_C</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
+          <t>Big Data Analytics, Data Mining, Machine Learning</t>
+        </is>
+      </c>
+      <c r="R7" s="8" t="inlineStr">
+        <is>
+          <t>ISE_S5_A, ISE_S5_B, ISE_S7_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
       <c r="A8" s="9" t="n">
         <v>4</v>
       </c>
@@ -869,13 +884,13 @@
         </is>
       </c>
       <c r="D8" s="11" t="n">
-        <v>16</v>
-      </c>
-      <c r="E8" s="9" t="n">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>13</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G8" s="9" t="n">
         <v>0</v>
@@ -887,35 +902,38 @@
         <v>0</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K8" s="9" t="n">
         <v>2</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O8" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="P8" s="12" t="inlineStr">
-        <is>
-          <t>Business Analytics, Cloud Computing, Information Security</t>
-        </is>
+      <c r="P8" s="9" t="n">
+        <v>2</v>
       </c>
       <c r="Q8" s="12" t="inlineStr">
         <is>
-          <t>CSBS_S5_A, ISE_S5_A, ISE_S5_B</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
+          <t>Big Data Analytics, Deep Learning, Physical Education</t>
+        </is>
+      </c>
+      <c r="R8" s="12" t="inlineStr">
+        <is>
+          <t>CSBS_S7_A, ISE_S7_A, ISE_S7_A,CSBS_S7_A, ISE_S7_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
@@ -932,51 +950,54 @@
       <c r="D9" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="E9" s="5" t="n">
-        <v>10</v>
+      <c r="E9" s="7" t="n">
+        <v>15</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="I9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="K9" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L9" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="M9" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="N9" s="5" t="n">
-        <v>3</v>
-      </c>
       <c r="O9" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>Advanced Database Systems, Artificial Intelligence, Big Data Analytics</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="P9" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>ISE_S7_A, ISE_S7_B</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
+          <t>Computer Networks, Data Structures, Data Structures Lab</t>
+        </is>
+      </c>
+      <c r="R9" s="8" t="inlineStr">
+        <is>
+          <t>CSBS_S3_B, ISE_S3_A, ISE_S3_C</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="9" t="n">
         <v>6</v>
       </c>
@@ -993,11 +1014,11 @@
       <c r="D10" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="E10" s="9" t="n">
-        <v>14</v>
+      <c r="E10" s="11" t="n">
+        <v>12</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G10" s="9" t="n">
         <v>0</v>
@@ -1009,35 +1030,38 @@
         <v>0</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>3</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N10" s="9" t="n">
         <v>2</v>
       </c>
       <c r="O10" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="P10" s="12" t="inlineStr">
-        <is>
-          <t>Cloud Computing, Data Structures, Probability and Statistics</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="P10" s="9" t="n">
+        <v>2</v>
       </c>
       <c r="Q10" s="12" t="inlineStr">
         <is>
-          <t>CSBS_S3_A, CSBS_S5_A, ISE_S5_A</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
+          <t>Business Analytics, Data Visualization, Operating Systems</t>
+        </is>
+      </c>
+      <c r="R10" s="12" t="inlineStr">
+        <is>
+          <t>CSBS_S5_A, ISE_S3_A, ISE_S3_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
@@ -1052,53 +1076,56 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>10</v>
+        <v>14</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>13</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N11" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="O11" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="O11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>Database Systems, Deep Learning Lab, Project Management</t>
-        </is>
+      <c r="P11" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>CSBS_S3_B, ISE_S7_A, ISE_S7_B</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
+          <t>Advanced Database Systems, Artificial Intelligence, Distributed Systems</t>
+        </is>
+      </c>
+      <c r="R11" s="8" t="inlineStr">
+        <is>
+          <t>ISE_S7_A, ISE_S7_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
       <c r="A12" s="9" t="n">
         <v>8</v>
       </c>
@@ -1113,16 +1140,16 @@
         </is>
       </c>
       <c r="D12" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="E12" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="E12" s="9" t="n">
-        <v>12</v>
-      </c>
       <c r="F12" s="9" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H12" s="9" t="n">
         <v>0</v>
@@ -1131,35 +1158,38 @@
         <v>0</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M12" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N12" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O12" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="P12" s="12" t="inlineStr">
-        <is>
-          <t>Big Data Analytics, Database Systems, Deep Learning Lab</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="P12" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="Q12" s="12" t="inlineStr">
         <is>
-          <t>CSBS_S3_A, CSBS_S7_A, ISE_S7_A</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="24" customHeight="1">
+          <t>Object Oriented Programming, Probability and Statistics</t>
+        </is>
+      </c>
+      <c r="R12" s="12" t="inlineStr">
+        <is>
+          <t>CSBS_S3_A, CSBS_S3_B, ISE_S3_C</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
       <c r="A13" s="5" t="n">
         <v>9</v>
       </c>
@@ -1174,53 +1204,56 @@
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>12</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="P13" s="8" t="inlineStr">
-        <is>
-          <t>Mathematics for Computing, Object Oriented Programming</t>
-        </is>
+      <c r="P13" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>ISE_S3_A, ISE_S3_B, ISE_S3_C</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
+          <t>Deep Learning Lab, Information Security, Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="R13" s="8" t="inlineStr">
+        <is>
+          <t>CSBS_S5_A, CSBS_S7_A, ISE_S7_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
       <c r="A14" s="9" t="n">
         <v>10</v>
       </c>
@@ -1235,53 +1268,56 @@
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>15</v>
-      </c>
-      <c r="E14" s="9" t="n">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>14</v>
       </c>
       <c r="F14" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="N14" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="M14" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="N14" s="9" t="n">
-        <v>3</v>
-      </c>
       <c r="O14" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="P14" s="12" t="inlineStr">
-        <is>
-          <t>Computer Networks, Operating Systems, Software Engineering</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="P14" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="Q14" s="12" t="inlineStr">
         <is>
-          <t>CSBS_S5_A, ISE_S3_A, ISE_S3_B</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1">
+          <t>Artificial Intelligence, Machine Learning Lab, Physical Education</t>
+        </is>
+      </c>
+      <c r="R14" s="12" t="inlineStr">
+        <is>
+          <t>CSBS_S5_A, ISE_S5_A, ISE_S5_A,CSBS_S5_A, ISE_S5_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
       <c r="A15" s="5" t="n">
         <v>11</v>
       </c>
@@ -1296,53 +1332,56 @@
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>8</v>
+        <v>16</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>18</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="I15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K15" s="5" t="n">
+      <c r="L15" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O15" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="L15" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="M15" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="N15" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="O15" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>Artificial Intelligence, Machine Learning Lab, Software Engineering</t>
-        </is>
+      <c r="P15" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="Q15" s="8" t="inlineStr">
         <is>
-          <t>CSBS_S5_A, ISE_S5_A, ISE_S5_B</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
+          <t>Data Structures, Database Management Systems, Object Oriented Programming</t>
+        </is>
+      </c>
+      <c r="R15" s="8" t="inlineStr">
+        <is>
+          <t>CSBS_S3_A, ISE_S3_A, ISE_S3_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
       <c r="A16" s="9" t="n">
         <v>12</v>
       </c>
@@ -1357,13 +1396,13 @@
         </is>
       </c>
       <c r="D16" s="11" t="n">
-        <v>21</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>17</v>
+        <v>16</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>18</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="G16" s="9" t="n">
         <v>0</v>
@@ -1372,38 +1411,41 @@
         <v>0</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L16" s="9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M16" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N16" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O16" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="P16" s="12" t="inlineStr">
-        <is>
-          <t>Deep Learning, Distributed Systems, Physical Education</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="P16" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="Q16" s="12" t="inlineStr">
         <is>
-          <t>CSBS_S7_A, ISE_S7_A, ISE_S7_A,CSBS_S7_A, ISE_S7_B</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
+          <t>Database Management Systems, Database Systems, Operating Systems</t>
+        </is>
+      </c>
+      <c r="R16" s="12" t="inlineStr">
+        <is>
+          <t>CSBS_S3_A, CSBS_S3_B, ISE_S3_C</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
       <c r="A17" s="5" t="n">
         <v>13</v>
       </c>
@@ -1418,34 +1460,34 @@
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>15</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L17" s="5" t="n">
         <v>2</v>
       </c>
       <c r="M17" s="5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N17" s="5" t="n">
         <v>2</v>
@@ -1453,18 +1495,21 @@
       <c r="O17" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>Business Intelligence, Natural Language Processing, Project Management</t>
-        </is>
+      <c r="P17" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>CSBS_S5_A, CSBS_S7_A, ISE_S7_B</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1">
+          <t>Communication Skills, Deep Learning Lab, Engineering Mathematics</t>
+        </is>
+      </c>
+      <c r="R17" s="8" t="inlineStr">
+        <is>
+          <t>CSBS_S1_A, CSBS_S1_B, ISE_S7_A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
       <c r="A18" s="9" t="n">
         <v>14</v>
       </c>
@@ -1479,13 +1524,13 @@
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>18</v>
-      </c>
-      <c r="E18" s="9" t="n">
-        <v>18</v>
+        <v>16</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>15</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G18" s="9" t="n">
         <v>0</v>
@@ -1497,35 +1542,38 @@
         <v>0</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L18" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M18" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N18" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O18" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="P18" s="12" t="inlineStr">
-        <is>
-          <t>Data Mining, Deep Learning, Web Technology</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="P18" s="9" t="n">
+        <v>4</v>
       </c>
       <c r="Q18" s="12" t="inlineStr">
         <is>
-          <t>CSBS_S7_A, ISE_S5_A, ISE_S5_B</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
+          <t>Cloud Computing, Software Engineering</t>
+        </is>
+      </c>
+      <c r="R18" s="12" t="inlineStr">
+        <is>
+          <t>CSBS_S5_A, ISE_S5_A, ISE_S5_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>15</v>
       </c>
@@ -1540,53 +1588,56 @@
         </is>
       </c>
       <c r="D19" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="F19" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="E19" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>0</v>
-      </c>
       <c r="G19" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M19" s="5" t="n">
         <v>2</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O19" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="P19" s="8" t="inlineStr">
-        <is>
-          <t>Communication Skills, Computer Organization, Object Oriented Programming</t>
-        </is>
+      <c r="P19" s="5" t="n">
+        <v>5</v>
       </c>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>CSBS_S1_A, CSBS_S1_B, CSBS_S3_B</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="24" customHeight="1">
+          <t>Distributed Systems, Machine Learning Lab, Project Management</t>
+        </is>
+      </c>
+      <c r="R19" s="8" t="inlineStr">
+        <is>
+          <t>CSBS_S7_A, ISE_S5_B, ISE_S7_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
       <c r="A20" s="9" t="n">
         <v>16</v>
       </c>
@@ -1601,13 +1652,13 @@
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>20</v>
+        <v>16</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>15</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G20" s="9" t="n">
         <v>0</v>
@@ -1619,35 +1670,38 @@
         <v>0</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K20" s="9" t="n">
         <v>3</v>
       </c>
       <c r="L20" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="M20" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="M20" s="9" t="n">
-        <v>3</v>
-      </c>
       <c r="N20" s="9" t="n">
         <v>1</v>
       </c>
       <c r="O20" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="P20" s="12" t="inlineStr">
-        <is>
-          <t>Data Structures, Database Management Systems, Digital Logic</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="P20" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="Q20" s="12" t="inlineStr">
         <is>
-          <t>CSBS_S1_B, ISE_S3_A, ISE_S3_B</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="24" customHeight="1">
+          <t>Deep Learning, Natural Language Processing, Project Management</t>
+        </is>
+      </c>
+      <c r="R20" s="12" t="inlineStr">
+        <is>
+          <t>ISE_S7_A, ISE_S7_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
       <c r="A21" s="5" t="n">
         <v>17</v>
       </c>
@@ -1662,53 +1716,56 @@
         </is>
       </c>
       <c r="D21" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="E21" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="E21" s="5" t="n">
-        <v>9</v>
-      </c>
       <c r="F21" s="5" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M21" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O21" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Data Structures Lab, Object Oriented Programming, Probability and Statistics</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="P21" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="Q21" s="8" t="inlineStr">
         <is>
-          <t>CSBS_S3_A, CSBS_S3_B, ISE_S3_A</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1">
+          <t>Data Structures, Data Structures Lab, Mathematics for Computing</t>
+        </is>
+      </c>
+      <c r="R21" s="8" t="inlineStr">
+        <is>
+          <t>ISE_S3_B, ISE_S3_C</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
       <c r="A22" s="9" t="n">
         <v>18</v>
       </c>
@@ -1723,14 +1780,14 @@
         </is>
       </c>
       <c r="D22" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E22" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="E22" s="9" t="n">
+      <c r="F22" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="F22" s="9" t="n">
-        <v>0</v>
-      </c>
       <c r="G22" s="9" t="n">
         <v>0</v>
       </c>
@@ -1741,35 +1798,38 @@
         <v>0</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L22" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M22" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N22" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O22" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="P22" s="12" t="inlineStr">
-        <is>
-          <t>Computer Networks, Natural Language Processing, Operating Systems</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="P22" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="Q22" s="12" t="inlineStr">
         <is>
-          <t>CSBS_S3_A, CSBS_S3_B, ISE_S7_A</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="24" customHeight="1">
+          <t>Information Security, Programming Fundamentals, Web Technology</t>
+        </is>
+      </c>
+      <c r="R22" s="12" t="inlineStr">
+        <is>
+          <t>CSBS_S1_B, ISE_S5_A, ISE_S5_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
       <c r="A23" s="5" t="n">
         <v>19</v>
       </c>
@@ -1784,53 +1844,56 @@
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="E23" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F23" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="F23" s="5" t="n">
-        <v>1</v>
-      </c>
       <c r="G23" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H23" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="K23" s="5" t="n">
-        <v>1</v>
-      </c>
       <c r="L23" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M23" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N23" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O23" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Computer Networks, Data Structures Lab, Database Management Systems</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="P23" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="Q23" s="8" t="inlineStr">
         <is>
-          <t>ISE_S3_B, ISE_S3_C</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="24" customHeight="1">
+          <t>Business Intelligence, Cloud Computing, Machine Learning</t>
+        </is>
+      </c>
+      <c r="R23" s="8" t="inlineStr">
+        <is>
+          <t>CSBS_S5_A, CSBS_S7_A, ISE_S5_A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
       <c r="A24" s="9" t="n">
         <v>20</v>
       </c>
@@ -1845,53 +1908,56 @@
         </is>
       </c>
       <c r="D24" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="E24" s="9" t="n">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>18</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G24" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="H24" s="9" t="n">
-        <v>0</v>
-      </c>
       <c r="I24" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K24" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="M24" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="L24" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="M24" s="9" t="n">
-        <v>4</v>
-      </c>
       <c r="N24" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O24" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="P24" s="12" t="inlineStr">
-        <is>
-          <t>Discrete Mathematics, Engineering Mathematics, Programming Fundamentals Lab</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="P24" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="Q24" s="12" t="inlineStr">
         <is>
+          <t>Computer Organization, Digital Logic, Programming Fundamentals Lab</t>
+        </is>
+      </c>
+      <c r="R24" s="12" t="inlineStr">
+        <is>
           <t>CSBS_S1_A, CSBS_S1_B</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="26" customHeight="1">
+    <row r="25" ht="25" customHeight="1">
       <c r="A25" s="13" t="inlineStr"/>
       <c r="B25" s="14" t="inlineStr">
         <is>
@@ -1904,47 +1970,50 @@
         </is>
       </c>
       <c r="D25" s="13" t="n">
-        <v>334</v>
+        <v>292</v>
       </c>
       <c r="E25" s="13" t="n">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="F25" s="13" t="n">
+        <v>234</v>
+      </c>
+      <c r="G25" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="G25" s="13" t="n">
+      <c r="H25" s="13" t="n">
         <v>39</v>
       </c>
-      <c r="H25" s="13" t="n">
+      <c r="I25" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="I25" s="13" t="n">
+      <c r="J25" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="J25" s="13" t="n">
-        <v>56</v>
-      </c>
       <c r="K25" s="13" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="L25" s="13" t="n">
+        <v>49</v>
+      </c>
+      <c r="M25" s="13" t="n">
+        <v>49</v>
+      </c>
+      <c r="N25" s="13" t="n">
         <v>54</v>
       </c>
-      <c r="M25" s="13" t="n">
-        <v>63</v>
-      </c>
-      <c r="N25" s="13" t="n">
-        <v>57</v>
-      </c>
       <c r="O25" s="13" t="n">
-        <v>57</v>
-      </c>
-      <c r="P25" s="14" t="inlineStr">
+        <v>46</v>
+      </c>
+      <c r="P25" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q25" s="14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q25" s="14" t="inlineStr">
+      <c r="R25" s="14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1952,9 +2021,10 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>